<commit_message>
Fix Excel formula generation and data fetching
- Fixed Yahoo Finance data fetching to properly transpose financial statements
- Updated Excel templates to embed formulas instead of static calculated values
- Added Model Inputs sections with key financial metrics in specific cells
- Fixed EV/EBITDA template to use Excel formulas like =4*B{i} for Target EV
- Fixed EV/Sales template to use Excel formulas for all calculations
- Updated sensitivity analysis to reference Summary sheet inputs
- Added debug script to verify financial data retrieval
- Now generates positive, realistic target prices for AAPL and MSFT

Co-Authored-By: robert.h@nobiliswealth.com <robert.h@nobiliswealth.com>
</commit_message>
<xml_diff>
--- a/output/AAPL_ev_ebitda_model.xlsx
+++ b/output/AAPL_ev_ebitda_model.xlsx
@@ -18,10 +18,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="$0.00"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -80,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -91,7 +90,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -457,15 +455,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -564,157 +562,226 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Valuation Analysis</t>
+          <t>Model Inputs</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Scenario</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>EV/EBITDA Multiple</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Target EV</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>Target Equity Value</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>Target Price</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>Upside/Downside</t>
-        </is>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>EBITDA (TTM):</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>134661000000</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Bear Case</t>
+          <t>Net Debt:</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>15</v>
-      </c>
-      <c r="C15" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" t="n">
-        <v>-76686000000</v>
-      </c>
-      <c r="E15" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="F15" s="4" t="n">
-        <v>-1.024315093986008</v>
+        <v>76686000000</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Base Case</t>
+          <t>Shares Outstanding:</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>18</v>
-      </c>
-      <c r="C16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" t="n">
-        <v>-76686000000</v>
-      </c>
-      <c r="E16" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="F16" s="4" t="n">
-        <v>-1.024315093986008</v>
+        <v>14935799649.32752</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>Current Price:</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>211.16</v>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Valuation Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>EV/EBITDA Multiple</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Target EV</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Target Equity Value</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Target Price</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Upside/Downside</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Bear Case</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>15</v>
+      </c>
+      <c r="C21">
+        <f>$B$14*B21</f>
+        <v/>
+      </c>
+      <c r="D21">
+        <f>C21-$B$15</f>
+        <v/>
+      </c>
+      <c r="E21">
+        <f>D21/$B$16</f>
+        <v/>
+      </c>
+      <c r="F21" s="4">
+        <f>(E21-$B$17)/$B$17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Base Case</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>18</v>
+      </c>
+      <c r="C22">
+        <f>$B$14*B22</f>
+        <v/>
+      </c>
+      <c r="D22">
+        <f>C22-$B$15</f>
+        <v/>
+      </c>
+      <c r="E22">
+        <f>D22/$B$16</f>
+        <v/>
+      </c>
+      <c r="F22" s="4">
+        <f>(E22-$B$17)/$B$17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>Bull Case</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B23" t="n">
         <v>22</v>
       </c>
-      <c r="C17" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" t="n">
-        <v>-76686000000</v>
-      </c>
-      <c r="E17" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="F17" s="4" t="n">
-        <v>-1.024315093986008</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="C23">
+        <f>$B$14*B23</f>
+        <v/>
+      </c>
+      <c r="D23">
+        <f>C23-$B$15</f>
+        <v/>
+      </c>
+      <c r="E23">
+        <f>D23/$B$16</f>
+        <v/>
+      </c>
+      <c r="F23" s="4">
+        <f>(E23-$B$17)/$B$17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>Current Multiple</t>
         </is>
       </c>
-      <c r="B18" t="n">
+      <c r="B24" t="n">
         <v>22.425</v>
       </c>
-      <c r="C18" t="n">
-        <v>0</v>
-      </c>
-      <c r="D18" t="n">
-        <v>-76686000000</v>
-      </c>
-      <c r="E18" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="F18" s="4" t="n">
-        <v>-1.024315093986008</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="C24">
+        <f>$B$14*B24</f>
+        <v/>
+      </c>
+      <c r="D24">
+        <f>C24-$B$15</f>
+        <v/>
+      </c>
+      <c r="E24">
+        <f>D24/$B$16</f>
+        <v/>
+      </c>
+      <c r="F24" s="4">
+        <f>(E24-$B$17)/$B$17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>Test Scenario</t>
         </is>
       </c>
-      <c r="B19" t="n">
+      <c r="B25" t="n">
         <v>19.5</v>
       </c>
-      <c r="C19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" t="n">
-        <v>-76686000000</v>
-      </c>
-      <c r="E19" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="F19" s="4" t="n">
-        <v>-1.024315093986008</v>
+      <c r="C25">
+        <f>$B$14*B25</f>
+        <v/>
+      </c>
+      <c r="D25">
+        <f>C25-$B$15</f>
+        <v/>
+      </c>
+      <c r="E25">
+        <f>D25/$B$16</f>
+        <v/>
+      </c>
+      <c r="F25" s="4">
+        <f>(E25-$B$17)/$B$17</f>
+        <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A13:F13"/>
+  <mergeCells count="4">
+    <mergeCell ref="A19:F19"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A13:B13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -730,17 +797,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="10" max="10"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -813,38 +880,49 @@
           <t>-10%</t>
         </is>
       </c>
-      <c r="B3" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="C3" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="D3" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="E3" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="F3" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="G3" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="H3" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="I3" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="J3" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="K3" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="L3" s="6" t="n">
-        <v>-5.134375246085518</v>
+      <c r="B3" s="6">
+        <f>(Summary.$B$14*(1+-0.1)*14-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="C3" s="6">
+        <f>(Summary.$B$14*(1+-0.1)*15-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="D3" s="6">
+        <f>(Summary.$B$14*(1+-0.1)*16-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="E3" s="6">
+        <f>(Summary.$B$14*(1+-0.1)*17-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="F3" s="6">
+        <f>(Summary.$B$14*(1+-0.1)*18-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="G3" s="6">
+        <f>(Summary.$B$14*(1+-0.1)*19-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="H3" s="6">
+        <f>(Summary.$B$14*(1+-0.1)*20-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="I3" s="6">
+        <f>(Summary.$B$14*(1+-0.1)*21-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="J3" s="6">
+        <f>(Summary.$B$14*(1+-0.1)*22-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="K3" s="6">
+        <f>(Summary.$B$14*(1+-0.1)*23-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="L3" s="6">
+        <f>(Summary.$B$14*(1+-0.1)*24-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -853,38 +931,49 @@
           <t>-5%</t>
         </is>
       </c>
-      <c r="B4" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="C4" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="D4" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="E4" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="F4" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="G4" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="H4" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="I4" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="J4" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="K4" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="L4" s="6" t="n">
-        <v>-5.134375246085518</v>
+      <c r="B4" s="6">
+        <f>(Summary.$B$14*(1+-0.05)*14-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="C4" s="6">
+        <f>(Summary.$B$14*(1+-0.05)*15-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="D4" s="6">
+        <f>(Summary.$B$14*(1+-0.05)*16-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="E4" s="6">
+        <f>(Summary.$B$14*(1+-0.05)*17-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="F4" s="6">
+        <f>(Summary.$B$14*(1+-0.05)*18-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="G4" s="6">
+        <f>(Summary.$B$14*(1+-0.05)*19-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="H4" s="6">
+        <f>(Summary.$B$14*(1+-0.05)*20-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="I4" s="6">
+        <f>(Summary.$B$14*(1+-0.05)*21-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="J4" s="6">
+        <f>(Summary.$B$14*(1+-0.05)*22-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="K4" s="6">
+        <f>(Summary.$B$14*(1+-0.05)*23-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="L4" s="6">
+        <f>(Summary.$B$14*(1+-0.05)*24-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -893,38 +982,49 @@
           <t>0%</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="C5" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="D5" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="E5" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="F5" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="G5" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="H5" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="I5" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="J5" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>-5.134375246085518</v>
+      <c r="B5" s="6">
+        <f>(Summary.$B$14*(1+0.0)*14-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="C5" s="6">
+        <f>(Summary.$B$14*(1+0.0)*15-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="D5" s="6">
+        <f>(Summary.$B$14*(1+0.0)*16-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="E5" s="6">
+        <f>(Summary.$B$14*(1+0.0)*17-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="F5" s="6">
+        <f>(Summary.$B$14*(1+0.0)*18-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="G5" s="6">
+        <f>(Summary.$B$14*(1+0.0)*19-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="H5" s="6">
+        <f>(Summary.$B$14*(1+0.0)*20-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="I5" s="6">
+        <f>(Summary.$B$14*(1+0.0)*21-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="J5" s="6">
+        <f>(Summary.$B$14*(1+0.0)*22-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="K5" s="6">
+        <f>(Summary.$B$14*(1+0.0)*23-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="L5" s="6">
+        <f>(Summary.$B$14*(1+0.0)*24-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -933,38 +1033,49 @@
           <t>5%</t>
         </is>
       </c>
-      <c r="B6" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="C6" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="D6" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="E6" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="F6" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="G6" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="H6" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="I6" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="J6" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="K6" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="L6" s="6" t="n">
-        <v>-5.134375246085518</v>
+      <c r="B6" s="6">
+        <f>(Summary.$B$14*(1+0.05)*14-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="C6" s="6">
+        <f>(Summary.$B$14*(1+0.05)*15-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="D6" s="6">
+        <f>(Summary.$B$14*(1+0.05)*16-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="E6" s="6">
+        <f>(Summary.$B$14*(1+0.05)*17-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="F6" s="6">
+        <f>(Summary.$B$14*(1+0.05)*18-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="G6" s="6">
+        <f>(Summary.$B$14*(1+0.05)*19-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="H6" s="6">
+        <f>(Summary.$B$14*(1+0.05)*20-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="I6" s="6">
+        <f>(Summary.$B$14*(1+0.05)*21-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="J6" s="6">
+        <f>(Summary.$B$14*(1+0.05)*22-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="K6" s="6">
+        <f>(Summary.$B$14*(1+0.05)*23-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="L6" s="6">
+        <f>(Summary.$B$14*(1+0.05)*24-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -973,38 +1084,49 @@
           <t>10%</t>
         </is>
       </c>
-      <c r="B7" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="E7" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="F7" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="G7" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="H7" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="I7" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="J7" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="K7" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="L7" s="6" t="n">
-        <v>-5.134375246085518</v>
+      <c r="B7" s="6">
+        <f>(Summary.$B$14*(1+0.1)*14-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="C7" s="6">
+        <f>(Summary.$B$14*(1+0.1)*15-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="D7" s="6">
+        <f>(Summary.$B$14*(1+0.1)*16-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="E7" s="6">
+        <f>(Summary.$B$14*(1+0.1)*17-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="F7" s="6">
+        <f>(Summary.$B$14*(1+0.1)*18-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="G7" s="6">
+        <f>(Summary.$B$14*(1+0.1)*19-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="H7" s="6">
+        <f>(Summary.$B$14*(1+0.1)*20-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="I7" s="6">
+        <f>(Summary.$B$14*(1+0.1)*21-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="J7" s="6">
+        <f>(Summary.$B$14*(1+0.1)*22-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="K7" s="6">
+        <f>(Summary.$B$14*(1+0.1)*23-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="L7" s="6">
+        <f>(Summary.$B$14*(1+0.1)*24-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -1013,38 +1135,49 @@
           <t>15%</t>
         </is>
       </c>
-      <c r="B8" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="D8" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="E8" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="F8" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="G8" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="H8" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="I8" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="J8" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="K8" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="L8" s="6" t="n">
-        <v>-5.134375246085518</v>
+      <c r="B8" s="6">
+        <f>(Summary.$B$14*(1+0.15)*14-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="C8" s="6">
+        <f>(Summary.$B$14*(1+0.15)*15-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="D8" s="6">
+        <f>(Summary.$B$14*(1+0.15)*16-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="E8" s="6">
+        <f>(Summary.$B$14*(1+0.15)*17-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="F8" s="6">
+        <f>(Summary.$B$14*(1+0.15)*18-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="G8" s="6">
+        <f>(Summary.$B$14*(1+0.15)*19-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="H8" s="6">
+        <f>(Summary.$B$14*(1+0.15)*20-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="I8" s="6">
+        <f>(Summary.$B$14*(1+0.15)*21-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="J8" s="6">
+        <f>(Summary.$B$14*(1+0.15)*22-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="K8" s="6">
+        <f>(Summary.$B$14*(1+0.15)*23-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="L8" s="6">
+        <f>(Summary.$B$14*(1+0.15)*24-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -1053,38 +1186,49 @@
           <t>20%</t>
         </is>
       </c>
-      <c r="B9" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="C9" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="E9" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="F9" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="G9" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="H9" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="I9" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="J9" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="K9" s="6" t="n">
-        <v>-5.134375246085518</v>
-      </c>
-      <c r="L9" s="6" t="n">
-        <v>-5.134375246085518</v>
+      <c r="B9" s="6">
+        <f>(Summary.$B$14*(1+0.2)*14-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="C9" s="6">
+        <f>(Summary.$B$14*(1+0.2)*15-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="D9" s="6">
+        <f>(Summary.$B$14*(1+0.2)*16-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="E9" s="6">
+        <f>(Summary.$B$14*(1+0.2)*17-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="F9" s="6">
+        <f>(Summary.$B$14*(1+0.2)*18-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="G9" s="6">
+        <f>(Summary.$B$14*(1+0.2)*19-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="H9" s="6">
+        <f>(Summary.$B$14*(1+0.2)*20-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="I9" s="6">
+        <f>(Summary.$B$14*(1+0.2)*21-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="J9" s="6">
+        <f>(Summary.$B$14*(1+0.2)*22-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="K9" s="6">
+        <f>(Summary.$B$14*(1+0.2)*23-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
+      </c>
+      <c r="L9" s="6">
+        <f>(Summary.$B$14*(1+0.2)*24-Summary.$B$15)/Summary.$B$16</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -1113,11 +1257,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="27" customWidth="1" min="1" max="1"/>
-    <col width="5" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1129,43 +1273,393 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="8" t="n">
-        <v>45565</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Tax Effect Of Unusual Items</t>
+        </is>
       </c>
       <c r="B3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="n">
-        <v>45199</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Tax Rate For Calcs</t>
+        </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>0.241</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="n">
-        <v>44834</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Normalized EBITDA</t>
+        </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>134661000000</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="n">
-        <v>44469</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Net Income From Continuing Operation Net Minority Interest</t>
+        </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>93736000000</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="n">
-        <v>44104</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Reconciled Depreciation</t>
+        </is>
       </c>
       <c r="B7" t="n">
-        <v/>
+        <v>11445000000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Reconciled Cost Of Revenue</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>210352000000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>134661000000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>EBIT</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>123216000000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Net Interest Income</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Interest Expense</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Interest Income</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Normalized Income</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>93736000000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Net Income From Continuing And Discontinued Operation</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>93736000000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Total Expenses</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>267819000000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Total Operating Income As Reported</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>123216000000</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Diluted Average Shares</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>15408095000</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Basic Average Shares</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>15343783000</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Diluted EPS</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>6.08</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Basic EPS</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>6.11</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Diluted NI Availto Com Stockholders</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>93736000000</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Net Income Common Stockholders</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>93736000000</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>93736000000</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Net Income Including Noncontrolling Interests</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>93736000000</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Net Income Continuous Operations</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>93736000000</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Tax Provision</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>29749000000</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Pretax Income</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>123485000000</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Other Income Expense</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>269000000</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Other Non Operating Income Expenses</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>269000000</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Net Non Operating Interest Income Expense</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Interest Expense Non Operating</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Interest Income Non Operating</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Operating Income</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>123216000000</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Operating Expense</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>57467000000</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Research And Development</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>31370000000</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Selling General And Administration</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>26097000000</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Gross Profit</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>180683000000</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Cost Of Revenue</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>210352000000</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Total Revenue</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>391035000000</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Operating Revenue</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>391035000000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>